<commit_message>
All features klar: checkin, checkout, chat till SQLite
</commit_message>
<xml_diff>
--- a/backend/logg.xlsx
+++ b/backend/logg.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -986,6 +986,9 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
+      <c r="J12" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1031,6 +1034,9 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
+      <c r="J13" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1076,6 +1082,9 @@
       <c r="I14" t="n">
         <v>38</v>
       </c>
+      <c r="J14" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1121,6 +1130,9 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
+      <c r="J15" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1166,6 +1178,9 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
+      <c r="J16" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1211,6 +1226,9 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
+      <c r="J17" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1256,6 +1274,9 @@
       <c r="I18" t="n">
         <v>0</v>
       </c>
+      <c r="J18" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1301,6 +1322,9 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
+      <c r="J19" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1346,6 +1370,9 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
+      <c r="J20" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -1413,6 +1440,9 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
+      <c r="J22" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1458,8 +1488,168 @@
       <c r="I23" t="n">
         <v>0</v>
       </c>
-      <c r="J23" t="n">
-        <v>0</v>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>18:43:27</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Södra Stenbocksgatan 116, Helsingborg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rasa Valatkeviviene</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0739916563</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>19:02:02</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Södra Stenbocksgatan 116, Helsingborg</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>19:02:08</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Södra Stenbocksgatan 116, Helsingborg</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mantas Vanagas</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0739916563</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>20:15:09</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Alegatan 16, Helsingborg</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>20:15:15</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Alegatan 16, Helsingborg</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mantas Vanagas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0739916563</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>21:10:58</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Alegatan 16, Helsingborg</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>21:11:14</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Alegatan 16, Helsingborg</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uppdatera hela systemet med alla nya funktioner och bugfixar
</commit_message>
<xml_diff>
--- a/backend/logg.xlsx
+++ b/backend/logg.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -986,9 +986,6 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1034,9 +1031,6 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1082,9 +1076,6 @@
       <c r="I14" t="n">
         <v>38</v>
       </c>
-      <c r="J14" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1130,9 +1121,6 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1178,9 +1166,6 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
-      <c r="J16" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1226,9 +1211,6 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1274,9 +1256,6 @@
       <c r="I18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1322,9 +1301,6 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1370,9 +1346,6 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -1440,9 +1413,6 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1600,9 +1570,6 @@
       <c r="I26" t="n">
         <v>0</v>
       </c>
-      <c r="J26" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1648,8 +1615,101 @@
       <c r="I27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" t="n">
-        <v>38</v>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Mantas Vanagas</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0739916563</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>08:47:10</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Eneborgsplatsen 3, Helsingborg</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>08:47:15</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Eneborgsplatsen 3, Helsingborg</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mantas Vanagas</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0739916563</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>08:48:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Eneborgsplatsen 3, Helsingborg</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>09:47:32</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Eneborgsplatsen 3, Helsingborg</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>59</v>
+      </c>
+      <c r="J29" t="n">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>